<commit_message>
Update: Excel template with corrected formatting
</commit_message>
<xml_diff>
--- a/Aprūpes lapas.xlsx
+++ b/Aprūpes lapas.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Pašaprūpes spēju novērtējums" sheetId="1" state="visible" r:id="rId3"/>
@@ -1022,7 +1022,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="73">
   <si>
     <t xml:space="preserve">Sociālā atbalsta centrs "Vaiņode"</t>
   </si>
@@ -1341,9 +1341,6 @@
       </rPr>
       <t xml:space="preserve"> — rakstām sarkani, cik ir. Ja zem 37°C — rakstām N.</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">38.6</t>
   </si>
   <si>
     <t xml:space="preserve">Higiēna</t>
@@ -2927,9 +2924,7 @@
         <v>44</v>
       </c>
       <c r="B10" s="26"/>
-      <c r="C10" s="27" t="s">
-        <v>45</v>
-      </c>
+      <c r="C10" s="27"/>
       <c r="D10" s="27"/>
       <c r="E10" s="27"/>
       <c r="F10" s="27"/>
@@ -2962,10 +2957,10 @@
     </row>
     <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="28" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" s="29" t="s">
         <v>46</v>
-      </c>
-      <c r="B11" s="29" t="s">
-        <v>47</v>
       </c>
       <c r="C11" s="25"/>
       <c r="D11" s="25"/>
@@ -3001,7 +2996,7 @@
     <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="28"/>
       <c r="B12" s="29" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C12" s="25"/>
       <c r="D12" s="25"/>
@@ -3037,7 +3032,7 @@
     <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="28"/>
       <c r="B13" s="29" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C13" s="25"/>
       <c r="D13" s="25"/>
@@ -3073,7 +3068,7 @@
     <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="28"/>
       <c r="B14" s="29" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C14" s="25"/>
       <c r="D14" s="25"/>
@@ -3109,7 +3104,7 @@
     <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="28"/>
       <c r="B15" s="29" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C15" s="25"/>
       <c r="D15" s="25"/>
@@ -3145,7 +3140,7 @@
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="28"/>
       <c r="B16" s="29" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C16" s="25"/>
       <c r="D16" s="25"/>
@@ -3181,7 +3176,7 @@
     <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="28"/>
       <c r="B17" s="29" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C17" s="25"/>
       <c r="D17" s="25"/>
@@ -3216,10 +3211,10 @@
     </row>
     <row r="18" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="28" t="s">
+        <v>53</v>
+      </c>
+      <c r="B18" s="29" t="s">
         <v>54</v>
-      </c>
-      <c r="B18" s="29" t="s">
-        <v>55</v>
       </c>
       <c r="C18" s="25"/>
       <c r="D18" s="25"/>
@@ -3255,7 +3250,7 @@
     <row r="19" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="28"/>
       <c r="B19" s="29" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C19" s="25"/>
       <c r="D19" s="25"/>
@@ -3291,7 +3286,7 @@
     <row r="20" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="28"/>
       <c r="B20" s="29" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C20" s="25"/>
       <c r="D20" s="25"/>
@@ -3326,10 +3321,10 @@
     </row>
     <row r="21" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="28" t="s">
+        <v>57</v>
+      </c>
+      <c r="B21" s="29" t="s">
         <v>58</v>
-      </c>
-      <c r="B21" s="29" t="s">
-        <v>59</v>
       </c>
       <c r="C21" s="25"/>
       <c r="D21" s="25"/>
@@ -3365,7 +3360,7 @@
     <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="28"/>
       <c r="B22" s="29" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C22" s="25"/>
       <c r="D22" s="25"/>
@@ -3401,7 +3396,7 @@
     <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="28"/>
       <c r="B23" s="29" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C23" s="25"/>
       <c r="D23" s="25"/>
@@ -3437,7 +3432,7 @@
     <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="28"/>
       <c r="B24" s="29" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C24" s="25"/>
       <c r="D24" s="25"/>
@@ -3472,10 +3467,10 @@
     </row>
     <row r="25" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="28" t="s">
+        <v>62</v>
+      </c>
+      <c r="B25" s="29" t="s">
         <v>63</v>
-      </c>
-      <c r="B25" s="29" t="s">
-        <v>64</v>
       </c>
       <c r="C25" s="25"/>
       <c r="D25" s="25"/>
@@ -3511,7 +3506,7 @@
     <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="28"/>
       <c r="B26" s="29" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C26" s="25"/>
       <c r="D26" s="25"/>
@@ -3546,7 +3541,7 @@
     </row>
     <row r="27" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="30" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B27" s="30"/>
       <c r="C27" s="25"/>
@@ -3582,7 +3577,7 @@
     </row>
     <row r="28" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="30" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B28" s="30"/>
       <c r="C28" s="25"/>
@@ -3618,7 +3613,7 @@
     </row>
     <row r="29" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="30" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B29" s="30"/>
       <c r="C29" s="25"/>
@@ -3654,7 +3649,7 @@
     </row>
     <row r="30" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="30" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B30" s="30"/>
       <c r="C30" s="25"/>
@@ -3690,7 +3685,7 @@
     </row>
     <row r="31" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="30" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B31" s="30"/>
       <c r="C31" s="25"/>
@@ -3726,7 +3721,7 @@
     </row>
     <row r="32" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="31" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B32" s="31"/>
       <c r="C32" s="32"/>
@@ -4040,7 +4035,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -4286,10 +4281,10 @@
     </row>
     <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="28" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" s="29" t="s">
         <v>46</v>
-      </c>
-      <c r="B5" s="29" t="s">
-        <v>47</v>
       </c>
       <c r="C5" s="25"/>
       <c r="D5" s="25"/>
@@ -4327,7 +4322,7 @@
     <row r="6" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="28"/>
       <c r="B6" s="29" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C6" s="25"/>
       <c r="D6" s="25"/>
@@ -4365,7 +4360,7 @@
     <row r="7" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="28"/>
       <c r="B7" s="29" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C7" s="25"/>
       <c r="D7" s="25"/>
@@ -4403,7 +4398,7 @@
     <row r="8" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="28"/>
       <c r="B8" s="29" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C8" s="25"/>
       <c r="D8" s="25"/>
@@ -4441,7 +4436,7 @@
     <row r="9" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="28"/>
       <c r="B9" s="29" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C9" s="25"/>
       <c r="D9" s="25"/>
@@ -4479,7 +4474,7 @@
     <row r="10" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="28"/>
       <c r="B10" s="29" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C10" s="25"/>
       <c r="D10" s="25"/>
@@ -4517,7 +4512,7 @@
     <row r="11" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="28"/>
       <c r="B11" s="29" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C11" s="25"/>
       <c r="D11" s="25"/>
@@ -4554,10 +4549,10 @@
     </row>
     <row r="12" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="28" t="s">
+        <v>53</v>
+      </c>
+      <c r="B12" s="29" t="s">
         <v>54</v>
-      </c>
-      <c r="B12" s="29" t="s">
-        <v>55</v>
       </c>
       <c r="C12" s="25"/>
       <c r="D12" s="25"/>
@@ -4595,7 +4590,7 @@
     <row r="13" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="28"/>
       <c r="B13" s="29" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C13" s="25"/>
       <c r="D13" s="25"/>
@@ -4633,7 +4628,7 @@
     <row r="14" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="28"/>
       <c r="B14" s="29" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C14" s="25"/>
       <c r="D14" s="25"/>
@@ -4670,10 +4665,10 @@
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="28" t="s">
+        <v>57</v>
+      </c>
+      <c r="B15" s="29" t="s">
         <v>58</v>
-      </c>
-      <c r="B15" s="29" t="s">
-        <v>59</v>
       </c>
       <c r="C15" s="25"/>
       <c r="D15" s="25"/>
@@ -4711,7 +4706,7 @@
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="28"/>
       <c r="B16" s="29" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C16" s="25"/>
       <c r="D16" s="25"/>
@@ -4749,7 +4744,7 @@
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="28"/>
       <c r="B17" s="29" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C17" s="25"/>
       <c r="D17" s="25"/>
@@ -4787,7 +4782,7 @@
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="28"/>
       <c r="B18" s="29" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C18" s="25"/>
       <c r="D18" s="25"/>
@@ -4824,10 +4819,10 @@
     </row>
     <row r="19" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="28" t="s">
+        <v>62</v>
+      </c>
+      <c r="B19" s="29" t="s">
         <v>63</v>
-      </c>
-      <c r="B19" s="29" t="s">
-        <v>64</v>
       </c>
       <c r="C19" s="25"/>
       <c r="D19" s="25"/>
@@ -4865,7 +4860,7 @@
     <row r="20" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="28"/>
       <c r="B20" s="29" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C20" s="25"/>
       <c r="D20" s="25"/>
@@ -4902,7 +4897,7 @@
     </row>
     <row r="21" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="30" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B21" s="30"/>
       <c r="C21" s="25"/>
@@ -4940,7 +4935,7 @@
     </row>
     <row r="22" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="30" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B22" s="30"/>
       <c r="C22" s="25"/>
@@ -4978,7 +4973,7 @@
     </row>
     <row r="23" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="30" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B23" s="30"/>
       <c r="C23" s="25"/>
@@ -5016,7 +5011,7 @@
     </row>
     <row r="24" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="30" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B24" s="30"/>
       <c r="C24" s="25"/>
@@ -5054,7 +5049,7 @@
     </row>
     <row r="25" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="30" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B25" s="30"/>
       <c r="C25" s="25"/>
@@ -5092,7 +5087,7 @@
     </row>
     <row r="26" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="31" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B26" s="31"/>
       <c r="C26" s="32"/>

</xml_diff>